<commit_message>
Add shower glass to Hank Fos budget
</commit_message>
<xml_diff>
--- a/estimates/7 St Elizabeth - Hank Fos - Master Bath/Hank_Fos_7_St_Elizabeth_Master_Bath.xlsx
+++ b/estimates/7 St Elizabeth - Hank Fos - Master Bath/Hank_Fos_7_St_Elizabeth_Master_Bath.xlsx
@@ -3087,11 +3087,15 @@
       <c r="A80" s="21" t="n"/>
       <c r="B80" s="22" t="inlineStr">
         <is>
-          <t>Engineering / Plans</t>
-        </is>
-      </c>
-      <c r="C80" s="23" t="n"/>
-      <c r="D80" s="23" t="n"/>
+          <t>Shower Glass Enclosure (68x34)</t>
+        </is>
+      </c>
+      <c r="C80" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="23" t="n">
+        <v>1800</v>
+      </c>
       <c r="E80" s="24">
         <f>IFERROR(C80+D80,0)</f>
         <v/>
@@ -3109,7 +3113,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I80" s="21" t="n"/>
+      <c r="I80" s="21" t="inlineStr">
+        <is>
+          <t>Semi-frameless; upgrade to full frameless adds ~$500</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="19" customHeight="1">
       <c r="A81" s="14" t="n"/>

</xml_diff>

<commit_message>
Rebuild Hank Fos budget — Justin's Numbers baseline, demo k, bidet pass-through
</commit_message>
<xml_diff>
--- a/estimates/7 St Elizabeth - Hank Fos - Master Bath/Hank_Fos_7_St_Elizabeth_Master_Bath.xlsx
+++ b/estimates/7 St Elizabeth - Hank Fos - Master Bath/Hank_Fos_7_St_Elizabeth_Master_Bath.xlsx
@@ -1894,14 +1894,14 @@
       <c r="A33" s="14" t="n"/>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Demo &amp; Haul Away</t>
         </is>
       </c>
       <c r="C33" s="16" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="E33" s="17">
         <f>IFERROR(C33+D33,0)</f>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="23" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="E34" s="24">
         <f>IFERROR(C34+D34,0)</f>
@@ -1958,14 +1958,14 @@
       <c r="A35" s="14" t="n"/>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>Tile Labor — Shower &amp; Toilet Room Walls (96" high)</t>
+          <t>Tile Labor — Shower &amp; Toilet Room Walls (96" high, niche)</t>
         </is>
       </c>
       <c r="C35" s="16" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>3000</v>
+        <v>3400</v>
       </c>
       <c r="E35" s="17">
         <f>IFERROR(C35+D35,0)</f>
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="D36" s="35" t="n">
         <v>0</v>
@@ -2003,9 +2003,8 @@
         <f>IFERROR(C36+D36,0)</f>
         <v/>
       </c>
-      <c r="F36" s="37">
-        <f>$F$6</f>
-        <v/>
+      <c r="F36" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="G36" s="38">
         <f>IFERROR(E36*(1+F36),0)</f>
@@ -2029,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="E37" s="17">
         <f>IFERROR(C37+D37,0)</f>
@@ -2058,7 +2057,7 @@
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="D38" s="35" t="n">
         <v>0</v>
@@ -2067,9 +2066,8 @@
         <f>IFERROR(C38+D38,0)</f>
         <v/>
       </c>
-      <c r="F38" s="37">
-        <f>$F$6</f>
-        <v/>
+      <c r="F38" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="G38" s="38">
         <f>IFERROR(E38*(1+F38),0)</f>
@@ -2093,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="E39" s="17">
         <f>IFERROR(C39+D39,0)</f>
@@ -2118,11 +2116,11 @@
       <c r="A40" s="33" t="n"/>
       <c r="B40" s="34" t="inlineStr">
         <is>
-          <t>Double Sink Vanity (Client Supplied)</t>
+          <t>Double Sink Vanity (Allowance)</t>
         </is>
       </c>
       <c r="C40" s="35" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D40" s="35" t="n">
         <v>0</v>
@@ -2131,9 +2129,8 @@
         <f>IFERROR(C40+D40,0)</f>
         <v/>
       </c>
-      <c r="F40" s="37">
-        <f>$F$6</f>
-        <v/>
+      <c r="F40" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="G40" s="38">
         <f>IFERROR(E40*(1+F40),0)</f>
@@ -2150,7 +2147,7 @@
       <c r="A41" s="33" t="n"/>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>Bidet Toilet (Allowance)</t>
+          <t>Bidet Toilet (Allowance — Pass-through)</t>
         </is>
       </c>
       <c r="C41" s="35" t="n">
@@ -2163,9 +2160,8 @@
         <f>IFERROR(C41+D41,0)</f>
         <v/>
       </c>
-      <c r="F41" s="37">
-        <f>$F$6</f>
-        <v/>
+      <c r="F41" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="G41" s="38">
         <f>IFERROR(E41*(1+F41),0)</f>
@@ -2314,7 +2310,7 @@
         </is>
       </c>
       <c r="C46" s="23" t="n">
-        <v>1200</v>
+        <v>700</v>
       </c>
       <c r="D46" s="23" t="n">
         <v>0</v>
@@ -2323,9 +2319,8 @@
         <f>IFERROR(C46+D46,0)</f>
         <v/>
       </c>
-      <c r="F46" s="18">
-        <f>$F$6</f>
-        <v/>
+      <c r="F46" s="18" t="n">
+        <v>0</v>
       </c>
       <c r="G46" s="19">
         <f>IFERROR(E46*(1+F46),0)</f>
@@ -2368,11 +2363,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I47" s="14" t="inlineStr">
-        <is>
-          <t>Mirror lights $500 allowance included in client price — add a separate allowance row if needed</t>
-        </is>
-      </c>
+      <c r="I47" s="14" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
@@ -3051,14 +3042,14 @@
       <c r="A79" s="14" t="n"/>
       <c r="B79" s="15" t="inlineStr">
         <is>
-          <t>Mirror Lights Allowance x2</t>
+          <t>Shower Glass Enclosure (68x34, semi-frameless)</t>
         </is>
       </c>
       <c r="C79" s="16" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="D79" s="16" t="n">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="E79" s="17">
         <f>IFERROR(C79+D79,0)</f>
@@ -3074,12 +3065,12 @@
       </c>
       <c r="H79" s="20" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I79" s="14" t="inlineStr">
         <is>
-          <t>Client selects fixtures</t>
+          <t>Upgrade to full frameless ~+$500</t>
         </is>
       </c>
     </row>
@@ -3087,22 +3078,21 @@
       <c r="A80" s="21" t="n"/>
       <c r="B80" s="22" t="inlineStr">
         <is>
-          <t>Shower Glass Enclosure (68x34)</t>
+          <t>Mirror Lights x2 (Allowance)</t>
         </is>
       </c>
       <c r="C80" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="D80" s="23" t="n">
         <v>0</v>
-      </c>
-      <c r="D80" s="23" t="n">
-        <v>1800</v>
       </c>
       <c r="E80" s="24">
         <f>IFERROR(C80+D80,0)</f>
         <v/>
       </c>
-      <c r="F80" s="18">
-        <f>$F$6</f>
-        <v/>
+      <c r="F80" s="18" t="n">
+        <v>0</v>
       </c>
       <c r="G80" s="19">
         <f>IFERROR(E80*(1+F80),0)</f>
@@ -3110,14 +3100,10 @@
       </c>
       <c r="H80" s="25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I80" s="21" t="inlineStr">
-        <is>
-          <t>Semi-frameless; upgrade to full frameless adds ~$500</t>
-        </is>
-      </c>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I80" s="21" t="n"/>
     </row>
     <row r="81" ht="19" customHeight="1">
       <c r="A81" s="14" t="n"/>
@@ -3637,274 +3623,124 @@
       </c>
     </row>
     <row r="6" ht="19" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
-        <is>
-          <t>Shower Tile</t>
-        </is>
-      </c>
-      <c r="B6" s="72" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="A6" s="72" t="n"/>
+      <c r="B6" s="72" t="n"/>
       <c r="C6" s="73" t="n"/>
       <c r="D6" s="74" t="n"/>
-      <c r="E6" s="75" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F6" s="74" t="inlineStr">
-        <is>
-          <t>Allowance</t>
-        </is>
-      </c>
-      <c r="G6" s="72" t="inlineStr">
-        <is>
-          <t>$2,000 client selects</t>
-        </is>
-      </c>
+      <c r="E6" s="75">
+        <f>IFERROR(C6*D6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="74" t="n"/>
+      <c r="G6" s="72" t="n"/>
     </row>
     <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="76" t="inlineStr">
-        <is>
-          <t>Floor Tile</t>
-        </is>
-      </c>
-      <c r="B7" s="76" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="A7" s="76" t="n"/>
+      <c r="B7" s="76" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="77" t="n"/>
-      <c r="E7" s="17" t="n">
-        <v>700</v>
-      </c>
-      <c r="F7" s="77" t="inlineStr">
-        <is>
-          <t>Allowance</t>
-        </is>
-      </c>
-      <c r="G7" s="76" t="inlineStr">
-        <is>
-          <t>$700 client selects</t>
-        </is>
-      </c>
+      <c r="E7" s="17">
+        <f>IFERROR(C7*D7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="77" t="n"/>
+      <c r="G7" s="76" t="n"/>
     </row>
     <row r="8" ht="19" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
-        <is>
-          <t>Bidet Toilet</t>
-        </is>
-      </c>
-      <c r="B8" s="72" t="inlineStr">
-        <is>
-          <t>Client TBD</t>
-        </is>
-      </c>
+      <c r="A8" s="72" t="n"/>
+      <c r="B8" s="72" t="n"/>
       <c r="C8" s="73" t="n"/>
       <c r="D8" s="74" t="n"/>
-      <c r="E8" s="75" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F8" s="74" t="inlineStr">
-        <is>
-          <t>Allowance</t>
-        </is>
-      </c>
-      <c r="G8" s="72" t="inlineStr">
-        <is>
-          <t>Client picks, $1k allowance</t>
-        </is>
-      </c>
+      <c r="E8" s="75">
+        <f>IFERROR(C8*D8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="74" t="n"/>
+      <c r="G8" s="72" t="n"/>
     </row>
     <row r="9" ht="19" customHeight="1">
-      <c r="A9" s="76" t="inlineStr">
-        <is>
-          <t>Mirror Lights x2</t>
-        </is>
-      </c>
-      <c r="B9" s="76" t="inlineStr">
-        <is>
-          <t>Client TBD</t>
-        </is>
-      </c>
+      <c r="A9" s="76" t="n"/>
+      <c r="B9" s="76" t="n"/>
       <c r="C9" s="16" t="n"/>
       <c r="D9" s="77" t="n"/>
-      <c r="E9" s="17" t="n">
-        <v>500</v>
-      </c>
-      <c r="F9" s="77" t="inlineStr">
-        <is>
-          <t>Allowance</t>
-        </is>
-      </c>
-      <c r="G9" s="76" t="inlineStr">
-        <is>
-          <t>$500 allowance</t>
-        </is>
-      </c>
+      <c r="E9" s="17">
+        <f>IFERROR(C9*D9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="77" t="n"/>
+      <c r="G9" s="76" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
-      <c r="A10" s="72" t="inlineStr">
-        <is>
-          <t>Sliding Closet Doors + Track</t>
-        </is>
-      </c>
-      <c r="B10" s="72" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="A10" s="72" t="n"/>
+      <c r="B10" s="72" t="n"/>
       <c r="C10" s="73" t="n"/>
       <c r="D10" s="74" t="n"/>
-      <c r="E10" s="75" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F10" s="74" t="inlineStr">
-        <is>
-          <t>Allowance</t>
-        </is>
-      </c>
-      <c r="G10" s="72" t="inlineStr">
-        <is>
-          <t>$1,200 allowance</t>
-        </is>
-      </c>
+      <c r="E10" s="75">
+        <f>IFERROR(C10*D10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="72" t="n"/>
     </row>
     <row r="11" ht="19" customHeight="1">
-      <c r="A11" s="76" t="inlineStr">
-        <is>
-          <t>Double Sink Vanity</t>
-        </is>
-      </c>
-      <c r="B11" s="76" t="inlineStr">
-        <is>
-          <t>Client Supplied</t>
-        </is>
-      </c>
+      <c r="A11" s="76" t="n"/>
+      <c r="B11" s="76" t="n"/>
       <c r="C11" s="16" t="n"/>
       <c r="D11" s="77" t="n"/>
-      <c r="E11" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="77" t="inlineStr">
-        <is>
-          <t>Client Supply</t>
-        </is>
-      </c>
-      <c r="G11" s="76" t="inlineStr">
-        <is>
-          <t>Client supplies</t>
-        </is>
-      </c>
+      <c r="E11" s="17">
+        <f>IFERROR(C11*D11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="77" t="n"/>
+      <c r="G11" s="76" t="n"/>
     </row>
     <row r="12" ht="19" customHeight="1">
-      <c r="A12" s="72" t="inlineStr">
-        <is>
-          <t>Faucets (2)</t>
-        </is>
-      </c>
-      <c r="B12" s="72" t="inlineStr">
-        <is>
-          <t>Client Supplied</t>
-        </is>
-      </c>
+      <c r="A12" s="72" t="n"/>
+      <c r="B12" s="72" t="n"/>
       <c r="C12" s="73" t="n"/>
       <c r="D12" s="74" t="n"/>
-      <c r="E12" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="74" t="inlineStr">
-        <is>
-          <t>Client Supply</t>
-        </is>
-      </c>
-      <c r="G12" s="72" t="inlineStr">
-        <is>
-          <t>Client supplies</t>
-        </is>
-      </c>
+      <c r="E12" s="75">
+        <f>IFERROR(C12*D12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="74" t="n"/>
+      <c r="G12" s="72" t="n"/>
     </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="A13" s="76" t="inlineStr">
-        <is>
-          <t>Shower Fixture</t>
-        </is>
-      </c>
-      <c r="B13" s="76" t="inlineStr">
-        <is>
-          <t>Client Supplied</t>
-        </is>
-      </c>
+      <c r="A13" s="76" t="n"/>
+      <c r="B13" s="76" t="n"/>
       <c r="C13" s="16" t="n"/>
       <c r="D13" s="77" t="n"/>
-      <c r="E13" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="77" t="inlineStr">
-        <is>
-          <t>Client Supply</t>
-        </is>
-      </c>
-      <c r="G13" s="76" t="inlineStr">
-        <is>
-          <t>Client supplies</t>
-        </is>
-      </c>
+      <c r="E13" s="17">
+        <f>IFERROR(C13*D13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="77" t="n"/>
+      <c r="G13" s="76" t="n"/>
     </row>
     <row r="14" ht="19" customHeight="1">
-      <c r="A14" s="72" t="inlineStr">
-        <is>
-          <t>Mirrors (2)</t>
-        </is>
-      </c>
-      <c r="B14" s="72" t="inlineStr">
-        <is>
-          <t>Client Supplied</t>
-        </is>
-      </c>
+      <c r="A14" s="72" t="n"/>
+      <c r="B14" s="72" t="n"/>
       <c r="C14" s="73" t="n"/>
       <c r="D14" s="74" t="n"/>
-      <c r="E14" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="74" t="inlineStr">
-        <is>
-          <t>Client Supply</t>
-        </is>
-      </c>
-      <c r="G14" s="72" t="inlineStr">
-        <is>
-          <t>Client supplies</t>
-        </is>
-      </c>
+      <c r="E14" s="75">
+        <f>IFERROR(C14*D14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="74" t="n"/>
+      <c r="G14" s="72" t="n"/>
     </row>
     <row r="15" ht="19" customHeight="1">
-      <c r="A15" s="76" t="inlineStr">
-        <is>
-          <t>Towel Bar + TP Holder</t>
-        </is>
-      </c>
-      <c r="B15" s="76" t="inlineStr">
-        <is>
-          <t>Client Supplied</t>
-        </is>
-      </c>
+      <c r="A15" s="76" t="n"/>
+      <c r="B15" s="76" t="n"/>
       <c r="C15" s="16" t="n"/>
       <c r="D15" s="77" t="n"/>
-      <c r="E15" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="77" t="inlineStr">
-        <is>
-          <t>Client Supply</t>
-        </is>
-      </c>
-      <c r="G15" s="76" t="inlineStr">
-        <is>
-          <t>Client supplies</t>
-        </is>
-      </c>
+      <c r="E15" s="17">
+        <f>IFERROR(C15*D15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="77" t="n"/>
+      <c r="G15" s="76" t="n"/>
     </row>
     <row r="16" ht="19" customHeight="1">
       <c r="A16" s="72" t="n"/>

</xml_diff>